<commit_message>
Supplementary Table 1: match the draft's residue-order naming
L100I+K103N in the Summary sheet and on its per-study tab, following the
same change in the manuscript.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper/submission/Supplementary-Table-1.xlsx
+++ b/paper/submission/Supplementary-Table-1.xlsx
@@ -21,7 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V106A+L234I" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V106M" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G190S" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K103N+L100I" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L100I+K103N" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K103N+P225H" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G190E" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="K103N+M230L" sheetId="19" state="visible" r:id="rId19"/>
@@ -1534,7 +1534,7 @@
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>K103N+L100I</t>
+          <t>L100I+K103N</t>
         </is>
       </c>
       <c r="C17" t="n">

</xml_diff>